<commit_message>
docs: add detection on parcels incluing roof objects and trees examples
</commit_message>
<xml_diff>
--- a/examples/detection/excel/excel_addresses_example.xlsx
+++ b/examples/detection/excel/excel_addresses_example.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/afryan/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{248FFFBF-6947-4F4D-BC90-0F98DCBF053D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1DEE377-149D-B640-9975-00F024C0CEEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17680" xr2:uid="{4C5EE341-500C-F94E-8B27-B0FC9A0037FE}"/>
+    <workbookView xWindow="1100" yWindow="820" windowWidth="28040" windowHeight="17440" xr2:uid="{5579C3DA-00F9-424E-B5A9-3EA9B5569F70}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
   <si>
-    <t>1 Rue De La Vau Saint-Jacques, 79200 Parthenay, France</t>
+    <t>238 Rue Pierre Mauroy</t>
   </si>
 </sst>
 </file>
@@ -409,12 +409,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1813D899-B066-884A-BD65-C73C98D7F122}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF1E5423-0AEE-1B45-AF6C-C99F38067095}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="40" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A1" t="s">

</xml_diff>